<commit_message>
Team Schedule capture as of 10/02/2026
</commit_message>
<xml_diff>
--- a/data/2026/cjsl/fall/albion-sc-brooklyn-b13-14-premier-williamsburg.xlsx
+++ b/data/2026/cjsl/fall/albion-sc-brooklyn-b13-14-premier-williamsburg.xlsx
@@ -214,7 +214,7 @@
       </c>
       <c r="I3" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>Rained Out</t>
         </is>
       </c>
     </row>
@@ -259,7 +259,7 @@
       </c>
       <c r="I4" s="0" t="inlineStr">
         <is>
-          <t/>
+          <t>Canceled</t>
         </is>
       </c>
     </row>

</xml_diff>